<commit_message>
Add sp_set_shop_rule for per-shop thresholds; seed Statement Collectables quarantine rule
Statement Collectables removes the price of sold items, so its rows without
a price are expected and must not fail the scrape health check.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentation/Statement_Data_Dictionary_Naming_Conventions_&_Lookup Tables.xlsx
+++ b/03_Documentation/Statement_Data_Dictionary_Naming_Conventions_&_Lookup Tables.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1324,6 +1324,33 @@
       <c r="E40" s="6" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>sp_set_shop_rule</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Creates or updates one shop's rules and thresholds</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>02_Stored_Procedures/10</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Writes ref_shop_rules</t>
         </is>
       </c>
     </row>
@@ -11786,7 +11813,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>One row per shop that behaves differently; the '*' row is the default. A NULL value falls back to the default.</t>
+          <t>One row per shop that behaves differently; the '*' row is the default. A NULL value falls back to the default. Set with CALL sp_set_shop_rule(shop, zero_price_means_sold, delist_grace_scrapes, min_count_ratio, max_quarantine_rate, max_duplicate_rate, max_field_empty_rate, min_expected_ratio, notes); NULL keeps the current value. Exception seeded: Statement Collectables max_quarantine_rate 0.3 (removes the price of sold items).</t>
         </is>
       </c>
     </row>
@@ -13946,7 +13973,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Verbs: load, validate, check, normalise, reconciled, run. Exceptions: sp_check_scrape_health, sp_run_pipeline.</t>
+          <t>Verbs: load, validate, check, normalise, reconciled, run, set. Exceptions: sp_check_scrape_health, sp_run_pipeline, sp_set_shop_rule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gold: give quarantined products a QUARANTINED status with the reason
Products that were scraped but never passed validation keep their NEW_LISTING
event and now get a status row instead of none.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentation/Statement_Data_Dictionary_Naming_Conventions_&_Lookup Tables.xlsx
+++ b/03_Documentation/Statement_Data_Dictionary_Naming_Conventions_&_Lookup Tables.xlsx
@@ -7883,7 +7883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8717,7 +8717,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>ACTIVE, ACTIVE_DISCOUNTED, PENDING_DELIST, SOLD.</t>
+          <t>ACTIVE, ACTIVE_DISCOUNTED, PENDING_DELIST, SOLD, QUARANTINED.</t>
         </is>
       </c>
     </row>
@@ -9067,81 +9067,89 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>quarantine_reason</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Why the product was quarantined.</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Bronze / Silver quarantine</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Latest reason; QUARANTINED products only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>gold_products_flat (01_DDL/06)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>One row per product: all attributes plus lifecycle status. Data Studio source.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>column_name</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>data_type</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>business_description</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>transformation_rules_&amp;_logic</t>
         </is>
       </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>product_id, url, title</t>
-        </is>
-      </c>
-      <c r="B63" s="6" t="inlineStr"/>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>Product.</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>fact_product_scrape</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>shop_name, region, city, latitude, longitude</t>
+          <t>product_id, url, title</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr"/>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Shop.</t>
+          <t>Product.</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>dim_shop</t>
+          <t>fact_product_scrape</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr"/>
@@ -9149,30 +9157,26 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>category, makers, primary_material</t>
+          <t>shop_name, region, city, latitude, longitude</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr"/>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Attributes.</t>
+          <t>Shop.</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>dim_category / dim_maker / dim_material</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>'-1' = unknown.</t>
-        </is>
-      </c>
+          <t>dim_shop</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>era, condition, dimensions</t>
+          <t>category, makers, primary_material</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr"/>
@@ -9183,7 +9187,7 @@
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>fact_product_scrape</t>
+          <t>dim_category / dim_maker / dim_material</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
@@ -9195,100 +9199,100 @@
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>status ... last_seen_at</t>
+          <t>era, condition, dimensions</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr"/>
       <c r="C67" s="6" t="inlineStr">
         <is>
+          <t>Attributes.</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>fact_product_scrape</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>'-1' = unknown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>status ... last_seen_at</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr"/>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
           <t>Lifecycle and prices.</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>gold_product_status</t>
         </is>
       </c>
-      <c r="E67" s="6" t="inlineStr">
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>status, sold_reason, sold_at, sold_price, current_price, current_available, first_listed_price, last_listed_price, markdown_count, total_markdown_pct, days_on_market, first_seen_at, last_seen_at.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>gold_market_products (01_DDL/07)</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>Base for the market views: one row per product with business labels. Products without price history are excluded.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>column_name</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>data_type</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>business_description</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr">
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>transformation_rules_&amp;_logic</t>
         </is>
       </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>product_id, url, title, shop_name</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="inlineStr"/>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>Product and shop.</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="inlineStr">
-        <is>
-          <t>gold_products_flat</t>
-        </is>
-      </c>
-      <c r="E72" s="6" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>region, city</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
+          <t>product_id, url, title, shop_name</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr"/>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Location.</t>
+          <t>Product and shop.</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -9296,16 +9300,12 @@
           <t>gold_products_flat</t>
         </is>
       </c>
-      <c r="E73" s="6" t="inlineStr">
-        <is>
-          <t>Empty becomes 'Unknown'.</t>
-        </is>
-      </c>
+      <c r="E73" s="6" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>region, city</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -9315,7 +9315,7 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Category.</t>
+          <t>Location.</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -9325,14 +9325,14 @@
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>NULL becomes 'Uncategorised'.</t>
+          <t>Empty becomes 'Unknown'.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>maker, material, era, condition</t>
+          <t>category</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
@@ -9342,58 +9342,62 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Attributes.</t>
+          <t>Category.</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>makers, primary_material, era, condition</t>
+          <t>gold_products_flat</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>'-1' or NULL becomes 'Unknown'.</t>
+          <t>NULL becomes 'Uncategorised'.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>status, sold_reason, sold_at</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr"/>
+          <t>maker, material, era, condition</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Lifecycle.</t>
+          <t>Attributes.</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>gold_products_flat</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr"/>
+          <t>makers, primary_material, era, condition</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>'-1' or NULL becomes 'Unknown'.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>is_sold</t>
-        </is>
-      </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>BOOL</t>
-        </is>
-      </c>
+          <t>status, sold_reason, sold_at</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr"/>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Status is SOLD.</t>
+          <t>Lifecycle.</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Derived</t>
+          <t>gold_products_flat</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr"/>
@@ -9401,7 +9405,7 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>is_sold</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -9411,7 +9415,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Status is ACTIVE, ACTIVE_DISCOUNTED or PENDING_DELIST.</t>
+          <t>Status is SOLD.</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -9424,57 +9428,57 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>sale_month</t>
+          <t>is_active</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>BOOL</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Month of sale.</t>
+          <t>Status is ACTIVE, ACTIVE_DISCOUNTED or PENDING_DELIST.</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>sold_at</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
-        <is>
-          <t>First day of the month.</t>
-        </is>
-      </c>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>sold_price</t>
+          <t>sale_month</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>NUMERIC</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Sale price.</t>
+          <t>Month of sale.</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>gold_products_flat</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr"/>
+          <t>sold_at</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>First day of the month.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>asking_price</t>
+          <t>sold_price</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
@@ -9484,24 +9488,20 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Current asking price.</t>
+          <t>Sale price.</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>last_listed_price</t>
-        </is>
-      </c>
-      <c r="E81" s="6" t="inlineStr">
-        <is>
-          <t>Last non-zero listed price.</t>
-        </is>
-      </c>
+          <t>gold_products_flat</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>first_listed_price, current_price</t>
+          <t>asking_price</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
@@ -9511,26 +9511,34 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Prices.</t>
+          <t>Current asking price.</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>gold_products_flat</t>
-        </is>
-      </c>
-      <c r="E82" s="6" t="inlineStr"/>
+          <t>last_listed_price</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Last non-zero listed price.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>markdown_count, total_markdown_pct, days_on_market</t>
-        </is>
-      </c>
-      <c r="B83" s="6" t="inlineStr"/>
+          <t>first_listed_price, current_price</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Discounting and velocity.</t>
+          <t>Prices.</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
@@ -9543,17 +9551,13 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>first_seen_at, last_seen_at</t>
-        </is>
-      </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
+          <t>markdown_count, total_markdown_pct, days_on_market</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr"/>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>First and last sighting.</t>
+          <t>Discounting and velocity.</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
@@ -9566,139 +9570,135 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
+          <t>first_seen_at, last_seen_at</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>First and last sighting.</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>gold_products_flat</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
           <t>listing_month</t>
         </is>
       </c>
-      <c r="B85" s="6" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
-      <c r="C85" s="6" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>Month first listed.</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>first_seen_at</t>
         </is>
       </c>
-      <c r="E85" s="6" t="inlineStr">
+      <c r="E86" s="6" t="inlineStr">
         <is>
           <t>First day of the month.</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="3" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
         <is>
           <t>Market insight views (01_DDL/07)</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="2" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>All built on gold_market_products. Regions cover the whole country.</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="4" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>view</t>
         </is>
       </c>
-      <c r="B89" s="4" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>grain</t>
         </is>
       </c>
-      <c r="C89" s="4" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>columns</t>
         </is>
       </c>
-      <c r="D89" s="4" t="inlineStr">
+      <c r="D90" s="4" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="E89" s="4" t="inlineStr">
+      <c r="E90" s="4" t="inlineStr">
         <is>
           <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>gold_sales</t>
-        </is>
-      </c>
-      <c r="B90" s="6" t="inlineStr">
-        <is>
-          <t>One row per sold product (national)</t>
-        </is>
-      </c>
-      <c r="C90" s="6" t="inlineStr">
-        <is>
-          <t>product_id, url, title, shop_name, region, city, category, maker, material, era, condition, sold_at, sale_month, sold_price, first_listed_price, total_markdown_pct, markdown_count, days_on_market, sold_reason</t>
-        </is>
-      </c>
-      <c r="D90" s="6" t="inlineStr">
-        <is>
-          <t>gold_market_products WHERE is_sold</t>
-        </is>
-      </c>
-      <c r="E90" s="6" t="inlineStr">
-        <is>
-          <t>Every sale in the country.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>gold_price_baseline</t>
+          <t>gold_sales</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>One row per segment</t>
+          <t>One row per sold product (national)</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>segment_type, segment, products, active_products, sold_products, sell_through_pct, asking_min, asking_p25, asking_median, asking_p75, asking_max, asking_mean, sold_p25, sold_median, sold_p75, sold_mean, median_days_on_market</t>
+          <t>product_id, url, title, shop_name, region, city, category, maker, material, era, condition, sold_at, sale_month, sold_price, first_listed_price, total_markdown_pct, markdown_count, days_on_market, sold_reason</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>gold_market_products</t>
+          <t>gold_market_products WHERE is_sold</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>segment_type: All products, Category, Material, Maker, Era, Condition, Region, Shop. Filter on segment_type.</t>
+          <t>Every sale in the country.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>gold_value_drivers</t>
+          <t>gold_price_baseline</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>One row per category x attribute</t>
+          <t>One row per segment</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>category, attribute_type, attribute, products, sold_products, median_asking_price, median_sold_price, category_products, category_median_asking_price, premium_pct, is_reliable</t>
+          <t>segment_type, segment, products, active_products, sold_products, sell_through_pct, asking_min, asking_p25, asking_median, asking_p75, asking_max, asking_mean, sold_p25, sold_median, sold_p75, sold_mean, median_days_on_market</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
@@ -9708,24 +9708,24 @@
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>premium_pct = attribute median / category median - 1. 'All categories' compares market-wide. is_reliable = 5+ products.</t>
+          <t>segment_type: All products, Category, Material, Maker, Era, Condition, Region, Shop. Filter on segment_type.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>gold_market_monthly</t>
+          <t>gold_value_drivers</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>One row per month x region x category</t>
+          <t>One row per category x attribute</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>month, region, category, new_listings, median_new_listing_price, sales, sold_value, median_sold_price, median_days_on_market, avg_markdown_pct_before_sale</t>
+          <t>category, attribute_type, attribute, products, sold_products, median_asking_price, median_sold_price, category_products, category_median_asking_price, premium_pct, is_reliable</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -9735,24 +9735,24 @@
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>Counts and values can be summed; medians apply to the row only.</t>
+          <t>premium_pct = attribute median / category median - 1. 'All categories' compares market-wide. is_reliable = 5+ products.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>gold_regional_demand</t>
+          <t>gold_market_monthly</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>One row per region</t>
+          <t>One row per month x region x category</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>region, shops, products_tracked, active_listings, active_stock_value, median_active_asking_price, sales, sales_last_90_days, sold_value, median_sold_price, median_days_on_market, sell_through_pct, share_of_national_sales_pct</t>
+          <t>month, region, category, new_listings, median_new_listing_price, sales, sold_value, median_sold_price, median_days_on_market, avg_markdown_pct_before_sale</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
@@ -9762,32 +9762,59 @@
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>All provinces.</t>
+          <t>Counts and values can be summed; medians apply to the row only.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
+          <t>gold_regional_demand</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>One row per region</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>region, shops, products_tracked, active_listings, active_stock_value, median_active_asking_price, sales, sales_last_90_days, sold_value, median_sold_price, median_days_on_market, sell_through_pct, share_of_national_sales_pct</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>gold_market_products</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>All provinces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
           <t>gold_shop_scorecard</t>
         </is>
       </c>
-      <c r="B95" s="6" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>One row per shop</t>
         </is>
       </c>
-      <c r="C95" s="6" t="inlineStr">
+      <c r="C96" s="6" t="inlineStr">
         <is>
           <t>shop_name, region, city, products_tracked, active_listings, discounted_listings, pending_delist, active_stock_value, median_active_asking_price, sales, sales_last_30_days, sales_last_90_days, sold_value, median_sold_price, median_days_on_market, avg_markdown_pct_before_sale, sell_through_pct, share_of_market_sales_pct</t>
         </is>
       </c>
-      <c r="D95" s="6" t="inlineStr">
+      <c r="D96" s="6" t="inlineStr">
         <is>
           <t>gold_market_products</t>
         </is>
       </c>
-      <c r="E95" s="6" t="inlineStr">
+      <c r="E96" s="6" t="inlineStr">
         <is>
           <t>Competitor benchmark.</t>
         </is>
@@ -11642,7 +11669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -13530,17 +13557,17 @@
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>MARKED_SOLD, ZERO_PRICE, DELISTED</t>
+          <t>QUARANTINED</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>Sold reason</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>Signal behind SOLD. Site signals take precedence over disappearance.</t>
+          <t>Scraped, but never passed validation (no price history). Keeps NEW_LISTING; never sold; excluded from gold_products_flat and the market views.</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr"/>
@@ -13549,17 +13576,17 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>HEALTHY, WARNING, FAILED</t>
+          <t>MARKED_SOLD, ZERO_PRICE, DELISTED</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>Scrape health</t>
+          <t>Sold reason</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>bronze_scrape_health.status and mon_scrape_runs.run_status.</t>
+          <t>Signal behind SOLD. Site signals take precedence over disappearance.</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr"/>
@@ -13568,21 +13595,40 @@
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>SUCCESS, PARTIAL, FAILED</t>
+          <t>HEALTHY, WARNING, FAILED</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>Scraper status</t>
+          <t>Scrape health</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>Run summary status.</t>
+          <t>bronze_scrape_health.status and mon_scrape_runs.run_status.</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr"/>
       <c r="E118" s="6" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>SUCCESS, PARTIAL, FAILED</t>
+        </is>
+      </c>
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>Scraper status</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="inlineStr">
+        <is>
+          <t>Run summary status.</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="inlineStr"/>
+      <c r="E119" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>